<commit_message>
Configuraciones a la app
</commit_message>
<xml_diff>
--- a/public/data/Registro de cursos.xlsx
+++ b/public/data/Registro de cursos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdlcastr\Line Pulse\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7024AA88-3786-4851-BEC0-5CD86ADE0871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148D6B51-0EEE-4978-83C4-01F0855E4A02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{568D8A14-5503-4228-893B-255CE258DEBD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="23">
   <si>
     <t>#Empleado</t>
   </si>
@@ -114,10 +114,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -158,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -170,6 +177,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -648,342 +657,468 @@
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>1003203</v>
-      </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
+      <c r="A3" s="5">
+        <v>1231908</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>4105793</v>
-      </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
+        <v>1220565</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>922501</v>
-      </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
+        <v>3004974</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="U5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="V5" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>1001749</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+      <c r="U6" s="6"/>
+      <c r="V6" s="6"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>29625</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
+      <c r="U7" s="6"/>
+      <c r="V7" s="6"/>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>4003495</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
+      <c r="U8" s="6"/>
+      <c r="V8" s="6"/>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>4023357</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+      <c r="O9" s="6"/>
+      <c r="P9" s="6"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+      <c r="U9" s="6"/>
+      <c r="V9" s="6"/>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>4067204</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+      <c r="U10" s="6"/>
+      <c r="V10" s="6"/>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>4083948</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
+      <c r="U11" s="6"/>
+      <c r="V11" s="6"/>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>4100076</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
-      <c r="T12" s="2"/>
-      <c r="U12" s="2"/>
-      <c r="V12" s="2"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="6"/>
+      <c r="U12" s="6"/>
+      <c r="V12" s="6"/>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>4101396</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="2"/>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
+      <c r="U13" s="6"/>
+      <c r="V13" s="6"/>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>4103260</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
-      <c r="U14" s="2"/>
-      <c r="V14" s="2"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="6"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="6"/>
+      <c r="U14" s="6"/>
+      <c r="V14" s="6"/>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>4104372</v>
       </c>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="6"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="6"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="6"/>
+      <c r="U15" s="6"/>
+      <c r="V15" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>